<commit_message>
Upgrade quotation tool to v2.0 with full analysis suite
- Multi-currency conversion: live rates (open.er-api.com) with built-in
  fallback for 30+ currencies; per-row currency support
- Supplier comparison: head-to-head metric table across all suppliers
- Part-level comparison: pivot of parts quoted by ≥2 suppliers with
  best/worst price highlighting and savings % calculation
- Discount column support: net price computed after discount
- 5-sheet Excel export: Overview (with bar chart), Supplier Comparison,
  Part Comparison (colour-coded), Line Items, Currency Rates
- CLI: --base-currency, --rates-file, --filter-supplier, --min-value,
  --top, --no-export, --list-sheets, --col-* overrides, --verbose
- Updated sample_quotation.xlsx with multi-currency and competitor rows

https://claude.ai/code/session_01MtyhoJGCr2jdPWtS3VzLwR
</commit_message>
<xml_diff>
--- a/sample_quotation.xlsx
+++ b/sample_quotation.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="44">
   <si>
     <t>Part No.</t>
   </si>
@@ -34,9 +34,15 @@
     <t>Currency</t>
   </si>
   <si>
+    <t>Discount</t>
+  </si>
+  <si>
     <t>Lead Time</t>
   </si>
   <si>
+    <t>Remarks</t>
+  </si>
+  <si>
     <t>V-2401</t>
   </si>
   <si>
@@ -109,22 +115,37 @@
     <t>FastBear Ltd</t>
   </si>
   <si>
+    <t>SinoValve Co.</t>
+  </si>
+  <si>
     <t>USD</t>
   </si>
   <si>
-    <t>2 weeks</t>
-  </si>
-  <si>
-    <t>4 weeks</t>
-  </si>
-  <si>
-    <t>1 week</t>
-  </si>
-  <si>
-    <t>3 weeks</t>
-  </si>
-  <si>
-    <t>6 weeks</t>
+    <t>CNY</t>
+  </si>
+  <si>
+    <t>2w</t>
+  </si>
+  <si>
+    <t>4w</t>
+  </si>
+  <si>
+    <t>1w</t>
+  </si>
+  <si>
+    <t>3w</t>
+  </si>
+  <si>
+    <t>6w</t>
+  </si>
+  <si>
+    <t>Preferred</t>
+  </si>
+  <si>
+    <t>High prio</t>
+  </si>
+  <si>
+    <t>Alt source</t>
   </si>
 </sst>
 </file>
@@ -456,10 +477,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -481,16 +502,22 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D2">
         <v>10</v>
@@ -499,21 +526,24 @@
         <v>45.5</v>
       </c>
       <c r="F2" t="s">
-        <v>31</v>
-      </c>
-      <c r="G2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+        <v>34</v>
+      </c>
+      <c r="G2">
+        <v>5</v>
+      </c>
+      <c r="H2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -522,21 +552,27 @@
         <v>1850</v>
       </c>
       <c r="F3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
+        <v>34</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D4">
         <v>50</v>
@@ -545,21 +581,24 @@
         <v>12.3</v>
       </c>
       <c r="F4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
+        <v>34</v>
+      </c>
+      <c r="G4">
+        <v>10</v>
+      </c>
+      <c r="H4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D5">
         <v>5</v>
@@ -568,21 +607,24 @@
         <v>110</v>
       </c>
       <c r="F5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5">
+        <v>5</v>
+      </c>
+      <c r="H5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
         <v>31</v>
-      </c>
-      <c r="G5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" t="s">
-        <v>29</v>
       </c>
       <c r="D6">
         <v>20</v>
@@ -591,21 +633,24 @@
         <v>8.75</v>
       </c>
       <c r="F6" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+        <v>34</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -614,21 +659,27 @@
         <v>3200</v>
       </c>
       <c r="F7" t="s">
-        <v>31</v>
-      </c>
-      <c r="G7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
+        <v>34</v>
+      </c>
+      <c r="G7">
+        <v>5</v>
+      </c>
+      <c r="H7" t="s">
+        <v>40</v>
+      </c>
+      <c r="I7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D8">
         <v>50</v>
@@ -637,21 +688,24 @@
         <v>10.8</v>
       </c>
       <c r="F8" t="s">
+        <v>34</v>
+      </c>
+      <c r="G8">
+        <v>10</v>
+      </c>
+      <c r="H8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" t="s">
         <v>31</v>
-      </c>
-      <c r="G8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" t="s">
-        <v>29</v>
       </c>
       <c r="D9">
         <v>100</v>
@@ -660,21 +714,24 @@
         <v>3.5</v>
       </c>
       <c r="F9" t="s">
-        <v>31</v>
-      </c>
-      <c r="G9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+        <v>34</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C10" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D10">
         <v>3</v>
@@ -683,21 +740,24 @@
         <v>275</v>
       </c>
       <c r="F10" t="s">
+        <v>34</v>
+      </c>
+      <c r="G10">
+        <v>5</v>
+      </c>
+      <c r="H10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
         <v>31</v>
-      </c>
-      <c r="G10" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" t="s">
-        <v>29</v>
       </c>
       <c r="D11">
         <v>15</v>
@@ -706,10 +766,100 @@
         <v>22</v>
       </c>
       <c r="F11" t="s">
-        <v>31</v>
-      </c>
-      <c r="G11" t="s">
+        <v>34</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12">
+        <v>10</v>
+      </c>
+      <c r="E12">
+        <v>280</v>
+      </c>
+      <c r="F12" t="s">
         <v>35</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12" t="s">
+        <v>39</v>
+      </c>
+      <c r="I12" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13">
+        <v>50</v>
+      </c>
+      <c r="E13">
+        <v>75</v>
+      </c>
+      <c r="F13" t="s">
+        <v>35</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13" t="s">
+        <v>36</v>
+      </c>
+      <c r="I13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+      <c r="E14">
+        <v>1650</v>
+      </c>
+      <c r="F14" t="s">
+        <v>35</v>
+      </c>
+      <c r="G14">
+        <v>5</v>
+      </c>
+      <c r="H14" t="s">
+        <v>37</v>
+      </c>
+      <c r="I14" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>